<commit_message>
Finish the ChatHealthyLib rename across the whole tree
The first rename commit covered what git tracks plus the design documents,
and reported itself complete. A sweep of every file in the tree found 194
still carrying the old name: the running copies under deploy/devops/, the
published schema under Website/schemas/, the brain and schema .bak files,
brain/BusinessArtifacts .pptx and .md, further .docx under
IdentityCertificatesAndAuthentications, the deployment-facts .xlsx
inventories and the FrontEnd DB matrices.

All of them now carry ChatHealthyLib / chathealthy_lib / chathealthy-lib.
The tree sweep is 0 of 3,631 files.

Verified locally: pipeline unit + regression 141 passed, enforcement suite
112 passed, chathealthy_lib imports, and build, deploy and promote all
start.

Three files could not be opened and are unverified: two Word ~$ lock files
under pipeline/ArchitectureDesignAndAudit/ and one corrupt .docx under
.vscode/.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/architecture/DevOpsBuildDeployAndEnvironmentManagement/deployment_facts_inventory_2026-06-26.xlsx
+++ b/architecture/DevOpsBuildDeployAndEnvironmentManagement/deployment_facts_inventory_2026-06-26.xlsx
@@ -3162,7 +3162,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/pyproject.toml</t>
+          <t>ChatHealthyLib/pyproject.toml</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/__init__.py</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/__init__.py</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/auth_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/auth_token.py</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/nonce.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/nonce.py</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/session_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/session_token.py</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/exceptions.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/exceptions.py</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/geo_extractor.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/geo_extractor.py</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/llm.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/llm.py</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/logging_service.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/logging_service.py</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/mongo_utilities.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/mongo_utilities.py</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/provider_embedding.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/provider_embedding.py</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/runtime_data_collections.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/runtime_data_collections.py</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/user/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/user/__init__.py</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_llm_facade.py</t>
+          <t>ChatHealthyLib/tests/test_llm_facade.py</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_logging_service_levels.py</t>
+          <t>ChatHealthyLib/tests/test_logging_service_levels.py</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_mongo_utilities_batch_size.py</t>
+          <t>ChatHealthyLib/tests/test_mongo_utilities_batch_size.py</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5054,12 +5054,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib</t>
+          <t>ChatHealthyLib</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib</t>
+          <t>ChatHealthyLib</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>{"src":"FrontEndApplicationLib"}</t>
+          <t>{"src":"ChatHealthyLib"}</t>
         </is>
       </c>
       <c r="H107" t="inlineStr"/>
@@ -10735,7 +10735,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -10778,7 +10778,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/pyproject.toml</t>
+          <t>ChatHealthyLib/pyproject.toml</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -10907,7 +10907,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/__init__.py</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/__init__.py</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -10993,7 +10993,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/auth_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/auth_token.py</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -11036,7 +11036,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/nonce.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/nonce.py</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/session_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/session_token.py</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -11122,7 +11122,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/exceptions.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/exceptions.py</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/geo_extractor.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/geo_extractor.py</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -11208,7 +11208,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/llm.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/llm.py</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -11251,7 +11251,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/logging_service.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/logging_service.py</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -11294,7 +11294,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/mongo_utilities.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/mongo_utilities.py</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -11337,7 +11337,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/provider_embedding.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/provider_embedding.py</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -11380,7 +11380,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/runtime_data_collections.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/runtime_data_collections.py</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/user/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/user/__init__.py</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -11466,7 +11466,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_llm_facade.py</t>
+          <t>ChatHealthyLib/tests/test_llm_facade.py</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -11509,7 +11509,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_logging_service_levels.py</t>
+          <t>ChatHealthyLib/tests/test_logging_service_levels.py</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -11552,7 +11552,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_mongo_utilities_batch_size.py</t>
+          <t>ChatHealthyLib/tests/test_mongo_utilities_batch_size.py</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -13699,12 +13699,12 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib</t>
+          <t>ChatHealthyLib</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib</t>
+          <t>ChatHealthyLib</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>{"src":"FrontEndApplicationLib"}</t>
+          <t>{"src":"ChatHealthyLib"}</t>
         </is>
       </c>
       <c r="H306" t="inlineStr"/>
@@ -14736,7 +14736,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
@@ -14779,7 +14779,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -14822,7 +14822,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -14865,7 +14865,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/pyproject.toml</t>
+          <t>ChatHealthyLib/pyproject.toml</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/__init__.py</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -14951,7 +14951,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/__init__.py</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/auth_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/auth_token.py</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
@@ -15037,7 +15037,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/nonce.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/nonce.py</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/session_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/session_token.py</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/exceptions.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/exceptions.py</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
@@ -15166,7 +15166,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/geo_extractor.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/geo_extractor.py</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
@@ -15209,7 +15209,7 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/llm.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/llm.py</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
@@ -15252,7 +15252,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/logging_service.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/logging_service.py</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
@@ -15295,7 +15295,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/mongo_utilities.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/mongo_utilities.py</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/provider_embedding.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/provider_embedding.py</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/runtime_data_collections.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/runtime_data_collections.py</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
@@ -15424,7 +15424,7 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/user/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/user/__init__.py</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
@@ -15467,7 +15467,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_llm_facade.py</t>
+          <t>ChatHealthyLib/tests/test_llm_facade.py</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -15510,7 +15510,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_logging_service_levels.py</t>
+          <t>ChatHealthyLib/tests/test_logging_service_levels.py</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -15553,7 +15553,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_mongo_utilities_batch_size.py</t>
+          <t>ChatHealthyLib/tests/test_mongo_utilities_batch_size.py</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
@@ -18173,12 +18173,12 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib</t>
+          <t>ChatHealthyLib</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib</t>
+          <t>ChatHealthyLib</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
@@ -18198,7 +18198,7 @@
       </c>
       <c r="G408" t="inlineStr">
         <is>
-          <t>{"src":"FrontEndApplicationLib"}</t>
+          <t>{"src":"ChatHealthyLib"}</t>
         </is>
       </c>
       <c r="H408" t="inlineStr"/>
@@ -23983,7 +23983,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
@@ -24026,7 +24026,7 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
         </is>
       </c>
       <c r="D544" t="inlineStr">
@@ -24069,7 +24069,7 @@
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
@@ -24112,7 +24112,7 @@
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/pyproject.toml</t>
+          <t>ChatHealthyLib/pyproject.toml</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
@@ -24155,7 +24155,7 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/__init__.py</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
@@ -24198,7 +24198,7 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/__init__.py</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
@@ -24241,7 +24241,7 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/auth_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/auth_token.py</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
@@ -24284,7 +24284,7 @@
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/nonce.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/nonce.py</t>
         </is>
       </c>
       <c r="D550" t="inlineStr">
@@ -24327,7 +24327,7 @@
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/session_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/session_token.py</t>
         </is>
       </c>
       <c r="D551" t="inlineStr">
@@ -24370,7 +24370,7 @@
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/exceptions.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/exceptions.py</t>
         </is>
       </c>
       <c r="D552" t="inlineStr">
@@ -24413,7 +24413,7 @@
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/geo_extractor.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/geo_extractor.py</t>
         </is>
       </c>
       <c r="D553" t="inlineStr">
@@ -24456,7 +24456,7 @@
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/llm.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/llm.py</t>
         </is>
       </c>
       <c r="D554" t="inlineStr">
@@ -24499,7 +24499,7 @@
       </c>
       <c r="C555" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/logging_service.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/logging_service.py</t>
         </is>
       </c>
       <c r="D555" t="inlineStr">
@@ -24542,7 +24542,7 @@
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/mongo_utilities.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/mongo_utilities.py</t>
         </is>
       </c>
       <c r="D556" t="inlineStr">
@@ -24585,7 +24585,7 @@
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/provider_embedding.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/provider_embedding.py</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
@@ -24628,7 +24628,7 @@
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/runtime_data_collections.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/runtime_data_collections.py</t>
         </is>
       </c>
       <c r="D558" t="inlineStr">
@@ -24671,7 +24671,7 @@
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/user/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/user/__init__.py</t>
         </is>
       </c>
       <c r="D559" t="inlineStr">
@@ -24714,7 +24714,7 @@
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_llm_facade.py</t>
+          <t>ChatHealthyLib/tests/test_llm_facade.py</t>
         </is>
       </c>
       <c r="D560" t="inlineStr">
@@ -24757,7 +24757,7 @@
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_logging_service_levels.py</t>
+          <t>ChatHealthyLib/tests/test_logging_service_levels.py</t>
         </is>
       </c>
       <c r="D561" t="inlineStr">
@@ -24800,7 +24800,7 @@
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_mongo_utilities_batch_size.py</t>
+          <t>ChatHealthyLib/tests/test_mongo_utilities_batch_size.py</t>
         </is>
       </c>
       <c r="D562" t="inlineStr">
@@ -27124,7 +27124,7 @@
       </c>
       <c r="C614" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
         </is>
       </c>
       <c r="D614" t="inlineStr">
@@ -27167,7 +27167,7 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
@@ -27210,7 +27210,7 @@
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">
@@ -27253,7 +27253,7 @@
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/pyproject.toml</t>
+          <t>ChatHealthyLib/pyproject.toml</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
@@ -27296,7 +27296,7 @@
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/__init__.py</t>
         </is>
       </c>
       <c r="D618" t="inlineStr">
@@ -27339,7 +27339,7 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/__init__.py</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
@@ -27382,7 +27382,7 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/auth_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/auth_token.py</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
@@ -27425,7 +27425,7 @@
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/nonce.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/nonce.py</t>
         </is>
       </c>
       <c r="D621" t="inlineStr">
@@ -27468,7 +27468,7 @@
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/session_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/session_token.py</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
@@ -27511,7 +27511,7 @@
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/exceptions.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/exceptions.py</t>
         </is>
       </c>
       <c r="D623" t="inlineStr">
@@ -27554,7 +27554,7 @@
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/geo_extractor.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/geo_extractor.py</t>
         </is>
       </c>
       <c r="D624" t="inlineStr">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/llm.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/llm.py</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
@@ -27640,7 +27640,7 @@
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/logging_service.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/logging_service.py</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
@@ -27683,7 +27683,7 @@
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/mongo_utilities.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/mongo_utilities.py</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
@@ -27726,7 +27726,7 @@
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/provider_embedding.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/provider_embedding.py</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
@@ -27769,7 +27769,7 @@
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/runtime_data_collections.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/runtime_data_collections.py</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
@@ -27812,7 +27812,7 @@
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/user/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/user/__init__.py</t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
@@ -27855,7 +27855,7 @@
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_llm_facade.py</t>
+          <t>ChatHealthyLib/tests/test_llm_facade.py</t>
         </is>
       </c>
       <c r="D631" t="inlineStr">
@@ -27898,7 +27898,7 @@
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_logging_service_levels.py</t>
+          <t>ChatHealthyLib/tests/test_logging_service_levels.py</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
@@ -27941,7 +27941,7 @@
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_mongo_utilities_batch_size.py</t>
+          <t>ChatHealthyLib/tests/test_mongo_utilities_batch_size.py</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
@@ -29795,7 +29795,7 @@
       </c>
       <c r="C675" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-003-Manage-Errors-design-v5.docx</t>
         </is>
       </c>
       <c r="D675" t="inlineStr">
@@ -29838,7 +29838,7 @@
       </c>
       <c r="C676" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v10.docx</t>
         </is>
       </c>
       <c r="D676" t="inlineStr">
@@ -29881,7 +29881,7 @@
       </c>
       <c r="C677" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
+          <t>ChatHealthyLib/architectureAndDesign/EPIC-003-F-005-Manage-Logging-design-v9.docx</t>
         </is>
       </c>
       <c r="D677" t="inlineStr">
@@ -29924,7 +29924,7 @@
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/pyproject.toml</t>
+          <t>ChatHealthyLib/pyproject.toml</t>
         </is>
       </c>
       <c r="D678" t="inlineStr">
@@ -29967,7 +29967,7 @@
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/__init__.py</t>
         </is>
       </c>
       <c r="D679" t="inlineStr">
@@ -30010,7 +30010,7 @@
       </c>
       <c r="C680" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/__init__.py</t>
         </is>
       </c>
       <c r="D680" t="inlineStr">
@@ -30053,7 +30053,7 @@
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/auth_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/auth_token.py</t>
         </is>
       </c>
       <c r="D681" t="inlineStr">
@@ -30096,7 +30096,7 @@
       </c>
       <c r="C682" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/nonce.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/nonce.py</t>
         </is>
       </c>
       <c r="D682" t="inlineStr">
@@ -30139,7 +30139,7 @@
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/session_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/session_token.py</t>
         </is>
       </c>
       <c r="D683" t="inlineStr">
@@ -30182,7 +30182,7 @@
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/exceptions.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/exceptions.py</t>
         </is>
       </c>
       <c r="D684" t="inlineStr">
@@ -30225,7 +30225,7 @@
       </c>
       <c r="C685" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/geo_extractor.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/geo_extractor.py</t>
         </is>
       </c>
       <c r="D685" t="inlineStr">
@@ -30268,7 +30268,7 @@
       </c>
       <c r="C686" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/llm.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/llm.py</t>
         </is>
       </c>
       <c r="D686" t="inlineStr">
@@ -30311,7 +30311,7 @@
       </c>
       <c r="C687" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/logging_service.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/logging_service.py</t>
         </is>
       </c>
       <c r="D687" t="inlineStr">
@@ -30354,7 +30354,7 @@
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/mongo_utilities.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/mongo_utilities.py</t>
         </is>
       </c>
       <c r="D688" t="inlineStr">
@@ -30397,7 +30397,7 @@
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/provider_embedding.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/provider_embedding.py</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
@@ -30440,7 +30440,7 @@
       </c>
       <c r="C690" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/runtime_data_collections.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/runtime_data_collections.py</t>
         </is>
       </c>
       <c r="D690" t="inlineStr">
@@ -30483,7 +30483,7 @@
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/user/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/user/__init__.py</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
@@ -30526,7 +30526,7 @@
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_llm_facade.py</t>
+          <t>ChatHealthyLib/tests/test_llm_facade.py</t>
         </is>
       </c>
       <c r="D692" t="inlineStr">
@@ -30569,7 +30569,7 @@
       </c>
       <c r="C693" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_logging_service_levels.py</t>
+          <t>ChatHealthyLib/tests/test_logging_service_levels.py</t>
         </is>
       </c>
       <c r="D693" t="inlineStr">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_mongo_utilities_batch_size.py</t>
+          <t>ChatHealthyLib/tests/test_mongo_utilities_batch_size.py</t>
         </is>
       </c>
       <c r="D694" t="inlineStr">
@@ -42220,7 +42220,7 @@
       </c>
       <c r="C962" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/__init__.py</t>
         </is>
       </c>
       <c r="D962" t="inlineStr">
@@ -42263,7 +42263,7 @@
       </c>
       <c r="C963" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/__init__.py</t>
         </is>
       </c>
       <c r="D963" t="inlineStr">
@@ -42306,7 +42306,7 @@
       </c>
       <c r="C964" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/auth_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/auth_token.py</t>
         </is>
       </c>
       <c r="D964" t="inlineStr">
@@ -42349,7 +42349,7 @@
       </c>
       <c r="C965" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/nonce.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/nonce.py</t>
         </is>
       </c>
       <c r="D965" t="inlineStr">
@@ -42392,7 +42392,7 @@
       </c>
       <c r="C966" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/authentication/session_token.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/authentication/session_token.py</t>
         </is>
       </c>
       <c r="D966" t="inlineStr">
@@ -42435,7 +42435,7 @@
       </c>
       <c r="C967" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/exceptions.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/exceptions.py</t>
         </is>
       </c>
       <c r="D967" t="inlineStr">
@@ -42478,7 +42478,7 @@
       </c>
       <c r="C968" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/geo_extractor.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/geo_extractor.py</t>
         </is>
       </c>
       <c r="D968" t="inlineStr">
@@ -42521,7 +42521,7 @@
       </c>
       <c r="C969" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/llm.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/llm.py</t>
         </is>
       </c>
       <c r="D969" t="inlineStr">
@@ -42564,7 +42564,7 @@
       </c>
       <c r="C970" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/logging_service.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/logging_service.py</t>
         </is>
       </c>
       <c r="D970" t="inlineStr">
@@ -42607,7 +42607,7 @@
       </c>
       <c r="C971" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/mongo_utilities.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/mongo_utilities.py</t>
         </is>
       </c>
       <c r="D971" t="inlineStr">
@@ -42650,7 +42650,7 @@
       </c>
       <c r="C972" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/provider_embedding.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/provider_embedding.py</t>
         </is>
       </c>
       <c r="D972" t="inlineStr">
@@ -42693,7 +42693,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/runtime_data_collections.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/runtime_data_collections.py</t>
         </is>
       </c>
       <c r="D973" t="inlineStr">
@@ -42736,7 +42736,7 @@
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/src/chathealthy_frontend_lib/user/__init__.py</t>
+          <t>ChatHealthyLib/src/chathealthy_lib/user/__init__.py</t>
         </is>
       </c>
       <c r="D974" t="inlineStr">
@@ -42779,7 +42779,7 @@
       </c>
       <c r="C975" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_llm_facade.py</t>
+          <t>ChatHealthyLib/tests/test_llm_facade.py</t>
         </is>
       </c>
       <c r="D975" t="inlineStr">
@@ -42822,7 +42822,7 @@
       </c>
       <c r="C976" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_logging_service_levels.py</t>
+          <t>ChatHealthyLib/tests/test_logging_service_levels.py</t>
         </is>
       </c>
       <c r="D976" t="inlineStr">
@@ -42865,7 +42865,7 @@
       </c>
       <c r="C977" t="inlineStr">
         <is>
-          <t>FrontEndApplicationLib/tests/test_mongo_utilities_batch_size.py</t>
+          <t>ChatHealthyLib/tests/test_mongo_utilities_batch_size.py</t>
         </is>
       </c>
       <c r="D977" t="inlineStr">

</xml_diff>